<commit_message>
pipeline for one regulation pdf
</commit_message>
<xml_diff>
--- a/Pravartiya/data/Links.xlsx
+++ b/Pravartiya/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -15,15 +15,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>Listed Companies</t>
-  </si>
-  <si>
-    <t>Circular-BSE</t>
-  </si>
-  <si>
-    <t>https://www.bseindia.com/corporates/CirularToListedComp.html</t>
   </si>
   <si>
     <t/>
@@ -32,10 +26,10 @@
     <t>SEBI</t>
   </si>
   <si>
-    <t>Informal Guidance</t>
+    <t>Regulations</t>
   </si>
   <si>
-    <t>https://www.sebi.gov.in/sebiweb/home/HomeAction.do?doListing=yes&amp;sid=2&amp;ssid=10&amp;smid=0</t>
+    <t>https://www.sebi.gov.in/sebiweb/home/HomeAction.do?doListingLegal=yes&amp;sid=1&amp;ssid=3&amp;smid=0</t>
   </si>
 </sst>
 </file>
@@ -132,16 +126,16 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
@@ -504,7 +498,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -532,11 +526,11 @@
       <c r="Z1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
+      <c r="A2" s="5" t="s">
+        <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>6</v>
+      <c r="B2" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -564,8 +558,8 @@
       <c r="Z2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="6"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -28573,7 +28567,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -28596,12 +28590,8 @@
       <c r="U2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>3</v>
-      </c>
+      <c r="A3" s="5"/>
+      <c r="B3" s="6"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>

</xml_diff>

<commit_message>
July newsletter except regulations
</commit_message>
<xml_diff>
--- a/Pravartiya/data/Links.xlsx
+++ b/Pravartiya/data/Links.xlsx
@@ -15,27 +15,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
   <si>
     <t>Listed Companies</t>
   </si>
   <si>
-    <t>Circular-BSE</t>
-  </si>
-  <si>
-    <t>https://www.bseindia.com/corporates/CirularToListedComp.html</t>
-  </si>
-  <si>
-    <t>Circular-NSE</t>
-  </si>
-  <si>
-    <t>https://www.nseindia.com/companies-listing/circular-for-listed-companies-equity-market</t>
+    <t/>
   </si>
   <si>
     <t>SEBI</t>
-  </si>
-  <si>
-    <t/>
   </si>
 </sst>
 </file>
@@ -132,10 +120,10 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
@@ -153,10 +141,10 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
@@ -473,7 +461,7 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="14" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="14" width="24.862142857142857" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="14" width="75.14785714285713" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="14" width="12.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="14" width="12.576428571428572" customWidth="1" bestFit="1"/>
@@ -504,7 +492,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -532,12 +520,8 @@
       <c r="Z1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>6</v>
-      </c>
+      <c r="A2" s="10"/>
+      <c r="B2" s="11"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -564,8 +548,8 @@
       <c r="Z2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="10"/>
+      <c r="B3" s="11"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -28573,7 +28557,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -28597,10 +28581,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
       <c r="A3" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -29013,7 +28997,7 @@
       <c r="T20" s="1"/>
       <c r="U20" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="1"/>
       <c r="B21" s="2"/>
       <c r="C21" s="1"/>

</xml_diff>

<commit_message>
july newsletter pravarthiya from server
</commit_message>
<xml_diff>
--- a/Pravartiya/data/Links.xlsx
+++ b/Pravartiya/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -15,15 +15,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="3">
   <si>
     <t>Listed Companies</t>
   </si>
   <si>
-    <t/>
+    <t>SEBI</t>
   </si>
   <si>
-    <t>SEBI</t>
+    <t/>
   </si>
 </sst>
 </file>
@@ -120,10 +120,10 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
@@ -141,10 +141,10 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
@@ -492,7 +492,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -519,9 +519,13 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="10"/>
-      <c r="B2" s="11"/>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>2</v>
+      </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -548,8 +552,8 @@
       <c r="Z2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="10"/>
-      <c r="B3" s="11"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -28553,12 +28557,8 @@
       <c r="U1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -28580,12 +28580,8 @@
       <c r="U2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>

</xml_diff>